<commit_message>
Brazil ENSO client table: two El Nino classes (strong >= 1.6, normal otherwise)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCxjZoAHXMLJTirXSfbmgL
</commit_message>
<xml_diff>
--- a/timeseries/output/enso/brazil_enso_client.xlsx
+++ b/timeseries/output/enso/brazil_enso_client.xlsx
@@ -188,12 +188,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$5:$A$9</f>
+              <f>'Robusta'!$A$5:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$D$5:$D$9</f>
+              <f>'Robusta'!$D$5:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -275,7 +275,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Robusta'!G30</f>
+              <f>'Robusta'!G29</f>
             </strRef>
           </tx>
           <spPr>
@@ -285,12 +285,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$31:$A$49</f>
+              <f>'Robusta'!$A$30:$A$48</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$G$31:$G$49</f>
+              <f>'Robusta'!$G$30:$G$48</f>
             </numRef>
           </val>
         </ser>
@@ -364,12 +364,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$5:$A$9</f>
+              <f>'Arabica'!$A$5:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$D$5:$D$9</f>
+              <f>'Arabica'!$D$5:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -451,7 +451,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Arabica'!G30</f>
+              <f>'Arabica'!G29</f>
             </strRef>
           </tx>
           <spPr>
@@ -461,12 +461,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$31:$A$49</f>
+              <f>'Arabica'!$A$30:$A$48</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$G$31:$G$49</f>
+              <f>'Arabica'!$G$30:$G$48</f>
             </numRef>
           </val>
         </ser>
@@ -509,7 +509,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="2880000"/>
@@ -531,7 +531,7 @@
     <from>
       <col>10</col>
       <colOff>0</colOff>
-      <row>29</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -558,7 +558,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="2880000"/>
@@ -580,7 +580,7 @@
     <from>
       <col>10</col>
       <colOff>0</colOff>
-      <row>29</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -890,7 +890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1008,196 +1008,196 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.7 to 1.5</t>
+          <t>0.5 to 1.5</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5.292335794870251</v>
+        <v>-1.471924624435547</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-1.869158878504673</v>
+        <v>-21.76470588235294</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>10.11904761904763</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-130.595238095238</v>
+        <v>-179.6785714285713</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.8261904761904724</v>
+        <v>0.7678571428571423</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2010/11, 2019/20, 2024/25</t>
+          <t>2010/11, 2015/16, 2019/20, 2024/25</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>El Nino weak</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.5 to 0.7</t>
+          <t>-0.7 to 0.5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-21.76470588235294</v>
+        <v>6.311212762825665</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.76470588235294</v>
+        <v>-0.6451612903225823</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-21.76470588235294</v>
+        <v>10.38961038961039</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-326.9285714285713</v>
+        <v>17.07142857142867</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.5928571428571416</v>
+        <v>-0.007142857142859782</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2013/14, 2014/15, 2020/21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-0.7 to 0.5</t>
+          <t>&lt;= -0.7</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>6.311212762825665</v>
+        <v>10.3783141585675</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.6451612903225823</v>
+        <v>-7.8125</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>10.38961038961039</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>17.07142857142867</v>
+        <v>18.67142857142858</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-0.007142857142859782</v>
+        <v>-0.1171428571428592</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2013/14, 2014/15, 2020/21</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+          <t>2008/09, 2009/10, 2011/12, 2012/13, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Year by year</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Crop year</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Index (RONI)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>ENSO class</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Robusta previous</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Robusta production</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Rain ES (mm)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Temp ES (°C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2008/09</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>La Nina</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>&lt;= -0.7</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>10.3783141585675</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>-7.8125</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>33.33333333333333</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>18.67142857142858</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>-0.1171428571428592</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2008/09, 2009/10, 2011/12, 2012/13, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Year by year</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Crop year</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Index (RONI)</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>ENSO class</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Robusta previous</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Robusta production</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Change %</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Rain ES (mm)</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Temp ES (°C)</t>
-        </is>
+      <c r="E30" s="3" t="n">
+        <v>11450</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>12800</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>11.79039301310043</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>942</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>24.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2008/09</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1206,7 +1206,7 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>-1.7</v>
+        <v>-1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1214,25 +1214,25 @@
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>11450</v>
+        <v>12800</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>12800</v>
+        <v>11800</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>11.79039301310043</v>
+        <v>-7.8125</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>942</v>
+        <v>1416</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>24.2</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2010/11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1241,33 +1241,33 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>-1</v>
+        <v>1.5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>12800</v>
+        <v>11800</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>11800</v>
+        <v>12700</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-7.8125</v>
+        <v>7.627118644067798</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1416</v>
+        <v>1093</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>23.9</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2010/11</t>
+          <t>2011/12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1276,33 +1276,33 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>1.5</v>
+        <v>-1.6</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>11800</v>
+        <v>12700</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>12700</v>
+        <v>14500</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>7.627118644067798</v>
+        <v>14.17322834645669</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1093</v>
+        <v>1344</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>24.4</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2011/12</t>
+          <t>2012/13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1311,7 +1311,7 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>-1.6</v>
+        <v>-1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1319,16 +1319,16 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>12700</v>
+        <v>14500</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>14500</v>
+        <v>15500</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>14.17322834645669</v>
+        <v>6.896551724137923</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>1344</v>
+        <v>1275</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>23.5</v>
@@ -1337,7 +1337,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2012/13</t>
+          <t>2013/14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1346,33 +1346,33 @@
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>-1</v>
+        <v>-0.6</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>14500</v>
+        <v>15500</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15500</v>
+        <v>15400</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>6.896551724137923</v>
+        <v>-0.6451612903225823</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>1275</v>
+        <v>996</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>23.5</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2013/14</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.4</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1389,25 +1389,25 @@
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>15500</v>
+        <v>15400</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>15400</v>
+        <v>17000</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.6451612903225823</v>
+        <v>10.38961038961039</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>996</v>
+        <v>1228</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>24.4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1416,33 +1416,33 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>-0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>15400</v>
+        <v>17000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17000</v>
+        <v>13300</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>10.38961038961039</v>
+        <v>-21.76470588235294</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>1228</v>
+        <v>823</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>24</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1451,33 +1451,33 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0.6</v>
+        <v>2.3</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>El Nino weak</t>
+          <t>El Nino strong</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>17000</v>
+        <v>13300</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13300</v>
+        <v>10500</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-21.76470588235294</v>
+        <v>-21.05263157894737</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>823</v>
+        <v>678</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>24.8</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2017/18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1486,33 +1486,33 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>2.3</v>
+        <v>-1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>El Nino strong</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>13300</v>
+        <v>10500</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>10500</v>
+        <v>12600</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>-21.05263157894737</v>
+        <v>20</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>678</v>
+        <v>1077</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>25.5</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2017/18</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>-1</v>
+        <v>-1.1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1529,25 +1529,25 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>10500</v>
+        <v>12600</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>12600</v>
+        <v>16800</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>20</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1077</v>
+        <v>1194</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1556,33 +1556,33 @@
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>-1.1</v>
+        <v>0.8</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>12600</v>
+        <v>16800</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>16800</v>
+        <v>18500</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>33.33333333333333</v>
+        <v>10.11904761904763</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>1194</v>
+        <v>1143</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>24.1</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1591,33 +1591,33 @@
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
-        <v>16800</v>
+        <v>18500</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>18500</v>
+        <v>20200</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>10.11904761904763</v>
+        <v>9.189189189189184</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>1143</v>
+        <v>1277</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>24.8</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1626,33 +1626,33 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>0.3</v>
+        <v>-1.5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>18500</v>
+        <v>20200</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>20200</v>
+        <v>21700</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>9.189189189189184</v>
+        <v>7.425742574257432</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1277</v>
+        <v>960</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>-1.5</v>
+        <v>-1.2</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1669,25 +1669,25 @@
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>20200</v>
+        <v>21700</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>21700</v>
+        <v>22800</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>7.425742574257432</v>
+        <v>5.069124423963123</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>960</v>
+        <v>1182</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>24.5</v>
+        <v>24.1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2023/24</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>-1.2</v>
+        <v>-1.1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1704,25 +1704,25 @@
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>21700</v>
+        <v>22800</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>22800</v>
+        <v>21400</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>5.069124423963123</v>
+        <v>-6.140350877192979</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>1182</v>
+        <v>1222</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>24.1</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2023/24</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1731,33 +1731,33 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>-1.1</v>
+        <v>1.4</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>22800</v>
+        <v>21400</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>21400</v>
+        <v>21000</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>-6.140350877192979</v>
+        <v>-1.869158878504673</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>1222</v>
+        <v>822</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>24.4</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1766,42 +1766,42 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>1.4</v>
+        <v>-1.1</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>21400</v>
+        <v>21000</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>21000</v>
+        <v>25000</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-1.869158878504673</v>
+        <v>19.04761904761905</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>822</v>
+        <v>1074</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>25.9</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2026/27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>USDA estimate</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>-1.1</v>
+        <v>-1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1809,51 +1809,16 @@
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>21000</v>
+        <v>25000</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>25000</v>
+        <v>24400</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>19.04761904761905</v>
-      </c>
-      <c r="H48" s="3" t="n">
-        <v>1074</v>
-      </c>
-      <c r="I48" s="3" t="n">
-        <v>24.7</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026/27</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>USDA estimate</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>La Nina</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F49" s="3" t="n">
-        <v>24400</v>
-      </c>
-      <c r="G49" s="3" t="n">
         <v>-2.400000000000002</v>
       </c>
-      <c r="H49" s="3" t="n"/>
-      <c r="I49" s="3" t="n"/>
+      <c r="H48" s="3" t="n"/>
+      <c r="I48" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1867,7 +1832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1985,14 +1950,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.7 to 1.5</t>
+          <t>0.5 to 1.5</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3.427613441101943</v>
+        <v>1.766420536590532</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>-15.49295774647888</v>
@@ -2001,180 +1966,180 @@
         <v>26.66666666666666</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-180.797619047619</v>
+        <v>-181.4642857142858</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.9404761904761934</v>
+        <v>0.8571428571428577</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2010/11, 2019/20, 2024/25</t>
+          <t>2010/11, 2015/16, 2019/20, 2024/25</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>El Nino weak</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.5 to 0.7</t>
+          <t>-0.7 to 0.5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-3.217158176943702</v>
+        <v>2.285064673488228</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-3.217158176943702</v>
+        <v>-10.76555023923444</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-3.217158176943702</v>
+        <v>18.33333333333334</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-183.4642857142858</v>
+        <v>-119.1309523809525</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.6071428571428612</v>
+        <v>0.1738095238095241</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2013/14, 2014/15, 2020/21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-0.7 to 0.5</t>
+          <t>&lt;= -0.7</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2.285064673488228</v>
+        <v>2.552827991539765</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-10.76555023923444</v>
+        <v>-26.76056338028169</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>18.33333333333334</v>
+        <v>46.47377938517179</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-119.1309523809525</v>
+        <v>-25.36428571428587</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.1738095238095241</v>
+        <v>-0.05285714285713894</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2013/14, 2014/15, 2020/21</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+          <t>2008/09, 2009/10, 2011/12, 2012/13, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Year by year</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Crop year</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Index (RONI)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>ENSO class</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Arabica previous</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Arabica production</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Rain MG (mm)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Temp MG (°C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2008/09</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>La Nina</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>&lt;= -0.7</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>2.552827991539765</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>-26.76056338028169</v>
-      </c>
-      <c r="F9" s="3" t="n">
+      <c r="E30" s="3" t="n">
+        <v>27650</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>40500</v>
+      </c>
+      <c r="G30" s="3" t="n">
         <v>46.47377938517179</v>
       </c>
-      <c r="G9" s="3" t="n">
-        <v>-25.36428571428587</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>-0.05285714285713894</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2008/09, 2009/10, 2011/12, 2012/13, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Year by year</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Crop year</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Index (RONI)</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>ENSO class</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Arabica previous</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Arabica production</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Change %</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Rain MG (mm)</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Temp MG (°C)</t>
-        </is>
+      <c r="H30" s="3" t="n">
+        <v>1296</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>20.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2008/09</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2183,7 +2148,7 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>-1.7</v>
+        <v>-1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2191,16 +2156,16 @@
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>27650</v>
+        <v>40500</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>40500</v>
+        <v>33000</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>46.47377938517179</v>
+        <v>-18.51851851851852</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1296</v>
+        <v>1521</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>20.9</v>
@@ -2209,7 +2174,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2010/11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2218,33 +2183,33 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>-1</v>
+        <v>1.5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>40500</v>
+        <v>33000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>33000</v>
+        <v>41800</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-18.51851851851852</v>
+        <v>26.66666666666666</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1521</v>
+        <v>1125</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>20.9</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2010/11</t>
+          <t>2011/12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2253,33 +2218,33 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>1.5</v>
+        <v>-1.6</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>33000</v>
+        <v>41800</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>41800</v>
+        <v>34700</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>26.66666666666666</v>
+        <v>-16.98564593301436</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1125</v>
+        <v>1383</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>21.3</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2011/12</t>
+          <t>2012/13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2288,7 +2253,7 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>-1.6</v>
+        <v>-1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2296,25 +2261,25 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>41800</v>
+        <v>34700</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>34700</v>
+        <v>42100</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-16.98564593301436</v>
+        <v>21.32564841498559</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>1383</v>
+        <v>1253</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2012/13</t>
+          <t>2013/14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2323,33 +2288,33 @@
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>-1</v>
+        <v>-0.6</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>34700</v>
+        <v>42100</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>42100</v>
+        <v>41800</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>21.32564841498559</v>
+        <v>-0.7125890736342066</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>1253</v>
+        <v>1260</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>20.7</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2013/14</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2358,7 +2323,7 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.4</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2366,25 +2331,25 @@
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>42100</v>
+        <v>41800</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>41800</v>
+        <v>37300</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-0.7125890736342066</v>
+        <v>-10.76555023923444</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1260</v>
+        <v>862</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>21.2</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2393,33 +2358,33 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>-0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>41800</v>
+        <v>37300</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>37300</v>
+        <v>36100</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-10.76555023923444</v>
+        <v>-3.217158176943702</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>862</v>
+        <v>1043</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2428,33 +2393,33 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0.6</v>
+        <v>2.3</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>El Nino weak</t>
+          <t>El Nino strong</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>37300</v>
+        <v>36100</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>36100</v>
+        <v>45600</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>-3.217158176943702</v>
+        <v>26.31578947368421</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>1043</v>
+        <v>1109</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2017/18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2463,33 +2428,33 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>2.3</v>
+        <v>-1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>El Nino strong</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>36100</v>
+        <v>45600</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>45600</v>
+        <v>39500</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>26.31578947368421</v>
+        <v>-13.37719298245614</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>1109</v>
+        <v>1018</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>22.2</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2017/18</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2498,7 +2463,7 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>-1</v>
+        <v>-1.1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2506,16 +2471,16 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>45600</v>
+        <v>39500</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>39500</v>
+        <v>49700</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-13.37719298245614</v>
+        <v>25.82278481012658</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1018</v>
+        <v>1158</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>21.5</v>
@@ -2524,7 +2489,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2533,33 +2498,33 @@
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>-1.1</v>
+        <v>0.8</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>39500</v>
+        <v>49700</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>49700</v>
+        <v>42000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>25.82278481012658</v>
+        <v>-15.49295774647888</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>1158</v>
+        <v>1231</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>21.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2568,33 +2533,33 @@
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
+        <v>42000</v>
+      </c>
+      <c r="F42" s="3" t="n">
         <v>49700</v>
       </c>
-      <c r="F42" s="3" t="n">
-        <v>42000</v>
-      </c>
       <c r="G42" s="3" t="n">
-        <v>-15.49295774647888</v>
+        <v>18.33333333333334</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>1231</v>
+        <v>1200</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>21.9</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2603,33 +2568,33 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>0.3</v>
+        <v>-1.5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>42000</v>
+        <v>49700</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>49700</v>
+        <v>36400</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>18.33333333333334</v>
+        <v>-26.76056338028169</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1200</v>
+        <v>860</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>21.6</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2638,7 +2603,7 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>-1.5</v>
+        <v>-1.2</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2646,25 +2611,25 @@
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>49700</v>
+        <v>36400</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>36400</v>
+        <v>39800</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>-26.76056338028169</v>
+        <v>9.340659340659329</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>860</v>
+        <v>1398</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>22.2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2023/24</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2673,7 +2638,7 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>-1.2</v>
+        <v>-1.1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2681,25 +2646,25 @@
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>36400</v>
+        <v>39800</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>39800</v>
+        <v>44900</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>9.340659340659329</v>
+        <v>12.81407035175879</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>1398</v>
+        <v>1210</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>21</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2023/24</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2708,33 +2673,33 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>-1.1</v>
+        <v>1.4</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>La Nina</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>39800</v>
+        <v>44900</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>44900</v>
+        <v>44500</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>12.81407035175879</v>
+        <v>-0.8908685968819552</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>1210</v>
+        <v>781</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>21.5</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2743,42 +2708,42 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>1.4</v>
+        <v>-1.1</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>44900</v>
+        <v>44500</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>44500</v>
+        <v>38000</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>-0.8908685968819552</v>
+        <v>-14.60674157303371</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>781</v>
+        <v>914</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>23.8</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2026/27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>USDA estimate</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>-1.1</v>
+        <v>-1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2786,51 +2751,16 @@
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>44500</v>
+        <v>38000</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>38000</v>
+        <v>47500</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>-14.60674157303371</v>
-      </c>
-      <c r="H48" s="3" t="n">
-        <v>914</v>
-      </c>
-      <c r="I48" s="3" t="n">
-        <v>22.4</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026/27</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>USDA estimate</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>La Nina</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>38000</v>
-      </c>
-      <c r="F49" s="3" t="n">
-        <v>47500</v>
-      </c>
-      <c r="G49" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="H49" s="3" t="n"/>
-      <c r="I49" s="3" t="n"/>
+      <c r="H48" s="3" t="n"/>
+      <c r="I48" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3940,7 +3870,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>El Nino weak</t>
+          <t>El Nino normal</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">

</xml_diff>

<commit_message>
Brazil ENSO client table: neutral band -0.5 to 0.5
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCxjZoAHXMLJTirXSfbmgL
</commit_message>
<xml_diff>
--- a/timeseries/output/enso/brazil_enso_client.xlsx
+++ b/timeseries/output/enso/brazil_enso_client.xlsx
@@ -1043,30 +1043,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-0.7 to 0.5</t>
+          <t>-0.5 to 0.5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>6.311212762825665</v>
+        <v>9.789399789399788</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.6451612903225823</v>
+        <v>9.189189189189184</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>10.38961038961039</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>17.07142857142867</v>
+        <v>102.5714285714287</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-0.007142857142859782</v>
+        <v>-0.1071428571428577</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2013/14, 2014/15, 2020/21</t>
+          <t>2014/15, 2020/21</t>
         </is>
       </c>
     </row>
@@ -1078,14 +1078,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>&lt;= -0.7</t>
+          <t>&lt;= -0.5</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>10.3783141585675</v>
+        <v>9.37618002685022</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>-7.8125</v>
@@ -1094,14 +1094,14 @@
         <v>33.33333333333333</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>18.67142857142858</v>
+        <v>2.980519480519661</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-0.1171428571428592</v>
+        <v>-0.08896103896103824</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2008/09, 2009/10, 2011/12, 2012/13, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
+          <t>2008/09, 2009/10, 2011/12, 2012/13, 2013/14, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
@@ -1985,14 +1985,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-0.7 to 0.5</t>
+          <t>-0.5 to 0.5</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2.285064673488228</v>
+        <v>3.783891547049445</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>-10.76555023923444</v>
@@ -2001,14 +2001,14 @@
         <v>18.33333333333334</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-119.1309523809525</v>
+        <v>-195.4642857142858</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.1738095238095241</v>
+        <v>0.3571428571428612</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2013/14, 2014/15, 2020/21</t>
+          <t>2014/15, 2020/21</t>
         </is>
       </c>
     </row>
@@ -2020,14 +2020,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>&lt;= -0.7</t>
+          <t>&lt;= -0.5</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2.552827991539765</v>
+        <v>2.255971894705767</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>-26.76056338028169</v>
@@ -2036,14 +2036,14 @@
         <v>46.47377938517179</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-25.36428571428587</v>
+        <v>-20.00974025974028</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-0.05285714285713894</v>
+        <v>-0.06558441558441075</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2008/09, 2009/10, 2011/12, 2012/13, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
+          <t>2008/09, 2009/10, 2011/12, 2012/13, 2013/14, 2017/18, 2018/19, 2021/22, 2022/23, 2023/24, 2025/26</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>La Nina</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">

</xml_diff>

<commit_message>
Brazil ENSO client table: 2015/16 counted as strong El Nino (peak 2.3 inside the marketing year)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCxjZoAHXMLJTirXSfbmgL
</commit_message>
<xml_diff>
--- a/timeseries/output/enso/brazil_enso_client.xlsx
+++ b/timeseries/output/enso/brazil_enso_client.xlsx
@@ -977,26 +977,26 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-21.05263157894737</v>
+        <v>-21.40866873065016</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-21.05263157894737</v>
+        <v>-21.76470588235294</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>-21.05263157894737</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-471.9285714285713</v>
+        <v>-399.4285714285713</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1.292857142857141</v>
+        <v>0.9428571428571395</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2015/16, 2016/17</t>
         </is>
       </c>
     </row>
@@ -1012,26 +1012,26 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-1.471924624435547</v>
+        <v>5.292335794870251</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.76470588235294</v>
+        <v>-1.869158878504673</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>10.11904761904763</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-179.6785714285713</v>
+        <v>-130.595238095238</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.7678571428571423</v>
+        <v>0.8261904761904724</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2010/11, 2015/16, 2019/20, 2024/25</t>
+          <t>2010/11, 2019/20, 2024/25</t>
         </is>
       </c>
     </row>
@@ -1416,11 +1416,11 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>0.6</v>
+        <v>2.3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>El Nino strong</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
@@ -1919,26 +1919,26 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>26.31578947368421</v>
+        <v>11.54931564837025</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>26.31578947368421</v>
+        <v>-3.217158176943702</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>26.31578947368421</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-117.4642857142858</v>
+        <v>-150.4642857142858</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.8071428571428605</v>
+        <v>0.7071428571428626</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2015/16, 2016/17</t>
         </is>
       </c>
     </row>
@@ -1954,10 +1954,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.766420536590532</v>
+        <v>3.427613441101943</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>-15.49295774647888</v>
@@ -1966,14 +1966,14 @@
         <v>26.66666666666666</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-181.4642857142858</v>
+        <v>-180.797619047619</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.8571428571428577</v>
+        <v>0.9404761904761934</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2010/11, 2015/16, 2019/20, 2024/25</t>
+          <t>2010/11, 2019/20, 2024/25</t>
         </is>
       </c>
     </row>
@@ -2358,11 +2358,11 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>0.6</v>
+        <v>2.3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>El Nino strong</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
@@ -3870,11 +3870,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>El Nino normal</t>
+          <t>El Nino strong</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.6</v>
+        <v>2.3</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>823</v>

</xml_diff>